<commit_message>
began on tech tree setting up files required etc
</commit_message>
<xml_diff>
--- a/Documentation/Tech tree.xlsx
+++ b/Documentation/Tech tree.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Documents\Final year uni\Comp-3000\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Documents\Final year uni\Comp-3000\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CC0F593-1490-409B-BAB7-83583ADF5AD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8C67B8E-B1E0-4B47-9F06-F97EA0A58A24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aspects of game" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="177">
   <si>
     <t>Core aspects</t>
   </si>
@@ -529,6 +529,36 @@
   </si>
   <si>
     <t>Capacity is double and can now contain 2 resources not 1</t>
+  </si>
+  <si>
+    <t>Implemented</t>
+  </si>
+  <si>
+    <t>Implemented2</t>
+  </si>
+  <si>
+    <t>Implemented3</t>
+  </si>
+  <si>
+    <t>Implemented4</t>
+  </si>
+  <si>
+    <t>Implemented5</t>
+  </si>
+  <si>
+    <t>Increase number of potential sniper towers</t>
+  </si>
+  <si>
+    <t>Adds guards on gate that fire at nearby enemies</t>
+  </si>
+  <si>
+    <t>Enemies take damage as they damage the depot</t>
+  </si>
+  <si>
+    <t>Can place mines</t>
+  </si>
+  <si>
+    <t>Increase depot health by 10%</t>
   </si>
 </sst>
 </file>
@@ -660,7 +690,22 @@
     <cellStyle name="60% - Accent6" xfId="2" builtinId="52"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="64">
+  <dxfs count="77">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -674,6 +719,9 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -683,6 +731,162 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -701,157 +905,22 @@
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -867,92 +936,105 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7936B949-188E-4582-8616-623FBF3C46A1}" name="Table1" displayName="Table1" ref="A1:D6" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7936B949-188E-4582-8616-623FBF3C46A1}" name="Table1" displayName="Table1" ref="A1:D6" totalsRowShown="0" headerRowDxfId="76" dataDxfId="75">
   <autoFilter ref="A1:D6" xr:uid="{7936B949-188E-4582-8616-623FBF3C46A1}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2EA6F07F-1C6E-40BA-AB5C-B295EB35CDCF}" name="Core aspects" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{194B2CAD-4A90-4E48-AEE8-DDC5F401A5C9}" name="Unit types" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{1448A4CC-616D-4E01-90A1-52101EAC6A7A}" name="Convoy types" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{B97AA103-9726-4AD2-A972-AE6976451B75}" name="Resources" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{2EA6F07F-1C6E-40BA-AB5C-B295EB35CDCF}" name="Core aspects" dataDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{194B2CAD-4A90-4E48-AEE8-DDC5F401A5C9}" name="Unit types" dataDxfId="73"/>
+    <tableColumn id="3" xr3:uid="{1448A4CC-616D-4E01-90A1-52101EAC6A7A}" name="Convoy types" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{B97AA103-9726-4AD2-A972-AE6976451B75}" name="Resources" dataDxfId="71"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}" name="Table4" displayName="Table4" ref="A1:L9" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:L9" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{273B543D-89B6-4955-A317-A6B9B4680CA3}" name="Defence upgrades" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{E2ECC974-9E12-4A07-BD63-BDCBEF1507C0}" name="Cost" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{2161316E-661A-4676-A677-BA66328341C0}" name="Pre-requsites" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{134C13E5-02FA-4F76-A06D-7102BADBA3D2}" name="Effect" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{CF1CB81C-0620-4735-BF49-5EF70D5A95D0}" name="Resource upgrades" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{D99D59BE-3DBC-4DC5-AC81-B6150EC1D1F4}" name="Cost2" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{02031DC9-8EF0-41F2-9B6C-598F6108A5A8}" name="Pre-requsites2" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{1680DD95-5CE0-4B9B-8549-ACF0137CB507}" name="Effect2" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{7E8E2876-1732-4CE0-B4F5-8E46B994DD1E}" name="Unit/Convoy unlocks" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{F2927B2C-24A0-4651-8D25-5F857B914BCE}" name="Cost3" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{DA739A9E-7639-4351-9932-0344E3EFE921}" name="Pre-requsites3" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{2CB92CE3-4985-4B3C-BB70-75B83BED998E}" name="Effect3" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}" name="Table4" displayName="Table4" ref="A1:O9" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+  <autoFilter ref="A1:O9" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{273B543D-89B6-4955-A317-A6B9B4680CA3}" name="Defence upgrades" dataDxfId="68"/>
+    <tableColumn id="5" xr3:uid="{E2ECC974-9E12-4A07-BD63-BDCBEF1507C0}" name="Cost" dataDxfId="67"/>
+    <tableColumn id="6" xr3:uid="{2161316E-661A-4676-A677-BA66328341C0}" name="Pre-requsites" dataDxfId="66"/>
+    <tableColumn id="12" xr3:uid="{134C13E5-02FA-4F76-A06D-7102BADBA3D2}" name="Effect" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{08607D56-09F1-4FA2-99AF-93D77D869DF9}" name="Implemented" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{CF1CB81C-0620-4735-BF49-5EF70D5A95D0}" name="Resource upgrades" dataDxfId="64"/>
+    <tableColumn id="8" xr3:uid="{D99D59BE-3DBC-4DC5-AC81-B6150EC1D1F4}" name="Cost2" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{02031DC9-8EF0-41F2-9B6C-598F6108A5A8}" name="Pre-requsites2" dataDxfId="62"/>
+    <tableColumn id="11" xr3:uid="{1680DD95-5CE0-4B9B-8549-ACF0137CB507}" name="Effect2" dataDxfId="61"/>
+    <tableColumn id="14" xr3:uid="{6C98FEC6-2863-482A-A27B-066A0999E0FB}" name="Implemented2" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{7E8E2876-1732-4CE0-B4F5-8E46B994DD1E}" name="Unit/Convoy unlocks" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{F2927B2C-24A0-4651-8D25-5F857B914BCE}" name="Cost3" dataDxfId="59"/>
+    <tableColumn id="10" xr3:uid="{DA739A9E-7639-4351-9932-0344E3EFE921}" name="Pre-requsites3" dataDxfId="58"/>
+    <tableColumn id="15" xr3:uid="{1806C71A-ADC9-4BB5-A94B-CBDCF0FD8313}" name="Effect3" dataDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{2CB92CE3-4985-4B3C-BB70-75B83BED998E}" name="Implemented3" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A9CB1332-57FC-4281-A975-E180D5843E29}" name="Table2" displayName="Table2" ref="A1:T6" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
-  <autoFilter ref="A1:T6" xr:uid="{A9CB1332-57FC-4281-A975-E180D5843E29}"/>
-  <tableColumns count="20">
-    <tableColumn id="2" xr3:uid="{E3DD0CDF-DC0D-4EB0-BEA2-5CE49EC8F866}" name="Generic upgrades" dataDxfId="41"/>
-    <tableColumn id="9" xr3:uid="{D795BCEF-0A20-4379-8C39-FA2DAF09421A}" name="Cost" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{D587DA64-F35B-4F32-B6F6-8E7BB1E63900}" name="Pre-requisites" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{4F232BF8-A260-479A-ACEC-63A224F97C46}" name="Effect" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{25E2217B-CC35-442F-87F5-43B6F7645DA5}" name="Basic infrantry unique upgrades" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{8C0715E7-FF65-417A-97C6-7BFE73531263}" name="Cost3" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{9FF16613-1C2D-4BB1-AB5A-3D830C82DC92}" name="Pre-requisites4" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{2034A85E-6909-4B73-B84A-8C8B031EE851}" name="Effect5" dataDxfId="34"/>
-    <tableColumn id="10" xr3:uid="{CCFAB2E6-3DF8-484A-B5C7-CEADB1D5A32D}" name="Scout unique upgrades" dataDxfId="33"/>
-    <tableColumn id="11" xr3:uid="{E2CFF5BF-4E7F-4723-BCD2-87DB4A1985D5}" name="Cost4" dataDxfId="32"/>
-    <tableColumn id="12" xr3:uid="{893B6115-0B13-4E43-99C3-E24E44F3F841}" name="Pre-requisites5" dataDxfId="31"/>
-    <tableColumn id="13" xr3:uid="{AD2BE189-025F-41D9-88E3-9F47A1E33C81}" name="Effect6" dataDxfId="30"/>
-    <tableColumn id="14" xr3:uid="{112DAB7A-25AB-4352-B02A-4C3400C87409}" name="Sniper unique upgrades" dataDxfId="29"/>
-    <tableColumn id="15" xr3:uid="{509A129B-88FA-4E7B-8193-F41864974FF7}" name="Cost5" dataDxfId="28"/>
-    <tableColumn id="16" xr3:uid="{1CFD16CF-9B96-461B-BA44-A4B5278D8678}" name="Pre-requisites6" dataDxfId="27"/>
-    <tableColumn id="17" xr3:uid="{9E59EF9D-9267-4AFC-A7A0-FE0D93235382}" name="Effect7" dataDxfId="26"/>
-    <tableColumn id="18" xr3:uid="{283492E4-882D-45FD-A134-10BDD63C01D3}" name="Melee unique upgrades" dataDxfId="25"/>
-    <tableColumn id="19" xr3:uid="{A63FDEF2-E4BB-4D35-8081-62BF6F91E6A6}" name="Cost6" dataDxfId="24"/>
-    <tableColumn id="20" xr3:uid="{FD236B57-46BD-4C72-910D-40EA2BEFE847}" name="Pre-requisites7" dataDxfId="23"/>
-    <tableColumn id="21" xr3:uid="{2620DB3A-6E53-4B05-BEB8-F5A55E804452}" name="Effect8" dataDxfId="22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A9CB1332-57FC-4281-A975-E180D5843E29}" name="Table2" displayName="Table2" ref="A1:Y6" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+  <autoFilter ref="A1:Y6" xr:uid="{A9CB1332-57FC-4281-A975-E180D5843E29}"/>
+  <tableColumns count="25">
+    <tableColumn id="2" xr3:uid="{E3DD0CDF-DC0D-4EB0-BEA2-5CE49EC8F866}" name="Generic upgrades" dataDxfId="54"/>
+    <tableColumn id="9" xr3:uid="{D795BCEF-0A20-4379-8C39-FA2DAF09421A}" name="Cost" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{D587DA64-F35B-4F32-B6F6-8E7BB1E63900}" name="Pre-requisites" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{4F232BF8-A260-479A-ACEC-63A224F97C46}" name="Effect" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{8AE9D933-FF62-449A-842E-5572F684C418}" name="Implemented" dataDxfId="9" dataCellStyle="60% - Accent4"/>
+    <tableColumn id="3" xr3:uid="{25E2217B-CC35-442F-87F5-43B6F7645DA5}" name="Basic infrantry unique upgrades" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{8C0715E7-FF65-417A-97C6-7BFE73531263}" name="Cost3" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{9FF16613-1C2D-4BB1-AB5A-3D830C82DC92}" name="Pre-requisites4" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{2034A85E-6909-4B73-B84A-8C8B031EE851}" name="Effect5" dataDxfId="47"/>
+    <tableColumn id="22" xr3:uid="{18C0C3D6-FC2F-4D61-8776-8A9C86198BFA}" name="Implemented2" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{CCFAB2E6-3DF8-484A-B5C7-CEADB1D5A32D}" name="Scout unique upgrades" dataDxfId="46"/>
+    <tableColumn id="11" xr3:uid="{E2CFF5BF-4E7F-4723-BCD2-87DB4A1985D5}" name="Cost4" dataDxfId="45"/>
+    <tableColumn id="12" xr3:uid="{893B6115-0B13-4E43-99C3-E24E44F3F841}" name="Pre-requisites5" dataDxfId="44"/>
+    <tableColumn id="13" xr3:uid="{AD2BE189-025F-41D9-88E3-9F47A1E33C81}" name="Effect6" dataDxfId="43"/>
+    <tableColumn id="23" xr3:uid="{C20328DE-0609-407C-AFCB-03B7812748D9}" name="Implemented3" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{112DAB7A-25AB-4352-B02A-4C3400C87409}" name="Sniper unique upgrades" dataDxfId="42"/>
+    <tableColumn id="15" xr3:uid="{509A129B-88FA-4E7B-8193-F41864974FF7}" name="Cost5" dataDxfId="41"/>
+    <tableColumn id="16" xr3:uid="{1CFD16CF-9B96-461B-BA44-A4B5278D8678}" name="Pre-requisites6" dataDxfId="40"/>
+    <tableColumn id="17" xr3:uid="{9E59EF9D-9267-4AFC-A7A0-FE0D93235382}" name="Effect7" dataDxfId="39"/>
+    <tableColumn id="24" xr3:uid="{FBB6ABB7-107D-48A8-ACA3-586EB6600CA8}" name="Implemented4" dataDxfId="6"/>
+    <tableColumn id="18" xr3:uid="{283492E4-882D-45FD-A134-10BDD63C01D3}" name="Melee unique upgrades" dataDxfId="38"/>
+    <tableColumn id="19" xr3:uid="{A63FDEF2-E4BB-4D35-8081-62BF6F91E6A6}" name="Cost6" dataDxfId="37"/>
+    <tableColumn id="20" xr3:uid="{FD236B57-46BD-4C72-910D-40EA2BEFE847}" name="Pre-requisites7" dataDxfId="36"/>
+    <tableColumn id="21" xr3:uid="{2620DB3A-6E53-4B05-BEB8-F5A55E804452}" name="Effect8" dataDxfId="35"/>
+    <tableColumn id="25" xr3:uid="{7073A254-5A8D-487B-ACBA-751FEA090B8F}" name="Implemented5" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6F54F13A-D763-4415-AF52-3251B521332F}" name="Table24" displayName="Table24" ref="A1:T4" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
-  <autoFilter ref="A1:T4" xr:uid="{6F54F13A-D763-4415-AF52-3251B521332F}"/>
-  <tableColumns count="20">
-    <tableColumn id="2" xr3:uid="{EB4E35EC-7A32-4043-AC4F-62F42A32D918}" name="Generic upgrades" dataDxfId="63"/>
-    <tableColumn id="3" xr3:uid="{B6D4A26B-841C-4651-B392-C413800BA49F}" name="Cost" dataDxfId="62"/>
-    <tableColumn id="5" xr3:uid="{92B340BF-E899-4C5E-A7EE-068FAE63D37E}" name="Pre-requisites" dataDxfId="61"/>
-    <tableColumn id="6" xr3:uid="{66255EC8-55E9-4791-B9A4-2658A7E89AB7}" name="Effect" dataDxfId="60"/>
-    <tableColumn id="7" xr3:uid="{8F1A242E-7826-4C78-A7FB-C0811E0DC38C}" name="Basic Convoy unique upgrades" dataDxfId="59"/>
-    <tableColumn id="8" xr3:uid="{880248A4-2E34-4E05-8EEE-19DAD8BA8D79}" name="Cost3" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{2AE87576-1799-432F-A7FD-846453B632F9}" name="Pre-requisites4" dataDxfId="57"/>
-    <tableColumn id="10" xr3:uid="{3D9BFB65-044E-46D6-BA79-605B541151F7}" name="Effect5" dataDxfId="56"/>
-    <tableColumn id="11" xr3:uid="{F2F0EDB8-2418-4120-A36E-6A799A139B44}" name="Armoured Convoy unique upgrades" dataDxfId="55"/>
-    <tableColumn id="12" xr3:uid="{74108871-80CF-4321-A45D-8AD943F641E5}" name="Cost4" dataDxfId="54"/>
-    <tableColumn id="13" xr3:uid="{528FAD47-5055-4C54-907C-AE802B24EE76}" name="Pre-requisites5" dataDxfId="53"/>
-    <tableColumn id="14" xr3:uid="{6FB45D9E-B476-4AAF-A885-1EE77EBB0A06}" name="Effect6" dataDxfId="52"/>
-    <tableColumn id="15" xr3:uid="{BA454E9F-DC7F-4486-A459-80E42B139783}" name="Medical Convoy unique upgrades" dataDxfId="51"/>
-    <tableColumn id="16" xr3:uid="{C32AC718-E815-45EA-97AD-9BBCB581C121}" name="Cost5" dataDxfId="50"/>
-    <tableColumn id="17" xr3:uid="{333DDDBD-0FA5-4B57-B26E-22C90DEAC453}" name="Pre-requisites6" dataDxfId="49"/>
-    <tableColumn id="18" xr3:uid="{DC44F460-C874-4BB4-946C-E222088CFB27}" name="Effect7" dataDxfId="48"/>
-    <tableColumn id="19" xr3:uid="{7EB0DD35-0EFD-4801-9E56-207D07409131}" name="Fast Convoy unique upgrades" dataDxfId="47"/>
-    <tableColumn id="20" xr3:uid="{242121C6-6B72-4769-BE45-504BC58B5446}" name="Cost6" dataDxfId="46"/>
-    <tableColumn id="21" xr3:uid="{1D20622B-A5D7-4451-BC95-05A11EC8C2F1}" name="Pre-requisites7" dataDxfId="45"/>
-    <tableColumn id="22" xr3:uid="{47D2D96E-45CA-4D18-9504-802D0C26A203}" name="Effect8" dataDxfId="44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6F54F13A-D763-4415-AF52-3251B521332F}" name="Table24" displayName="Table24" ref="A1:Y4" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+  <autoFilter ref="A1:Y4" xr:uid="{6F54F13A-D763-4415-AF52-3251B521332F}"/>
+  <tableColumns count="25">
+    <tableColumn id="2" xr3:uid="{EB4E35EC-7A32-4043-AC4F-62F42A32D918}" name="Generic upgrades" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{B6D4A26B-841C-4651-B392-C413800BA49F}" name="Cost" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{92B340BF-E899-4C5E-A7EE-068FAE63D37E}" name="Pre-requisites" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{66255EC8-55E9-4791-B9A4-2658A7E89AB7}" name="Effect" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{2948CF41-8302-4123-845E-240AC7F118B4}" name="Implemented" dataDxfId="4" dataCellStyle="60% - Accent4"/>
+    <tableColumn id="7" xr3:uid="{8F1A242E-7826-4C78-A7FB-C0811E0DC38C}" name="Basic Convoy unique upgrades" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{880248A4-2E34-4E05-8EEE-19DAD8BA8D79}" name="Cost3" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{2AE87576-1799-432F-A7FD-846453B632F9}" name="Pre-requisites4" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{3D9BFB65-044E-46D6-BA79-605B541151F7}" name="Effect5" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{FD82BA05-8A8E-4A4F-B060-96D26ADA1450}" name="Implemented2" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{F2F0EDB8-2418-4120-A36E-6A799A139B44}" name="Armoured Convoy unique upgrades" dataDxfId="24"/>
+    <tableColumn id="12" xr3:uid="{74108871-80CF-4321-A45D-8AD943F641E5}" name="Cost4" dataDxfId="23"/>
+    <tableColumn id="13" xr3:uid="{528FAD47-5055-4C54-907C-AE802B24EE76}" name="Pre-requisites5" dataDxfId="22"/>
+    <tableColumn id="14" xr3:uid="{6FB45D9E-B476-4AAF-A885-1EE77EBB0A06}" name="Effect6" dataDxfId="21"/>
+    <tableColumn id="23" xr3:uid="{81360CD7-893D-485D-89AD-B56D5C8C9B8C}" name="Implemented3" dataDxfId="2"/>
+    <tableColumn id="15" xr3:uid="{BA454E9F-DC7F-4486-A459-80E42B139783}" name="Medical Convoy unique upgrades" dataDxfId="20"/>
+    <tableColumn id="16" xr3:uid="{C32AC718-E815-45EA-97AD-9BBCB581C121}" name="Cost5" dataDxfId="19"/>
+    <tableColumn id="17" xr3:uid="{333DDDBD-0FA5-4B57-B26E-22C90DEAC453}" name="Pre-requisites6" dataDxfId="18"/>
+    <tableColumn id="18" xr3:uid="{DC44F460-C874-4BB4-946C-E222088CFB27}" name="Effect7" dataDxfId="17"/>
+    <tableColumn id="24" xr3:uid="{489DBCB6-36A9-4651-A748-9DCF7ED10EC4}" name="Implemented4" dataDxfId="1" dataCellStyle="60% - Accent4"/>
+    <tableColumn id="19" xr3:uid="{7EB0DD35-0EFD-4801-9E56-207D07409131}" name="Fast Convoy unique upgrades" dataDxfId="16"/>
+    <tableColumn id="20" xr3:uid="{242121C6-6B72-4769-BE45-504BC58B5446}" name="Cost6" dataDxfId="15"/>
+    <tableColumn id="21" xr3:uid="{1D20622B-A5D7-4451-BC95-05A11EC8C2F1}" name="Pre-requisites7" dataDxfId="14"/>
+    <tableColumn id="22" xr3:uid="{47D2D96E-45CA-4D18-9504-802D0C26A203}" name="Effect8" dataDxfId="13"/>
+    <tableColumn id="25" xr3:uid="{09417E2C-43AB-44A9-8F24-5ADC7305B330}" name="Implemented5" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1325,24 +1407,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7C1AE8C-0057-4B1D-8955-2B721776BB0B}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="28.140625" customWidth="1"/>
-    <col min="5" max="5" width="27.85546875" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="27.85546875" customWidth="1"/>
-    <col min="8" max="8" width="28.28515625" customWidth="1"/>
-    <col min="9" max="9" width="25.28515625" customWidth="1"/>
-    <col min="10" max="10" width="26.28515625" customWidth="1"/>
-    <col min="11" max="11" width="28.28515625" customWidth="1"/>
-    <col min="12" max="12" width="15.140625" customWidth="1"/>
+    <col min="4" max="5" width="28.140625" customWidth="1"/>
+    <col min="6" max="6" width="27.85546875" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
+    <col min="8" max="8" width="27.85546875" customWidth="1"/>
+    <col min="9" max="10" width="28.28515625" customWidth="1"/>
+    <col min="11" max="11" width="25.28515625" customWidth="1"/>
+    <col min="12" max="12" width="26.28515625" customWidth="1"/>
+    <col min="13" max="14" width="28.28515625" customWidth="1"/>
+    <col min="15" max="15" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>24</v>
       </c>
@@ -1356,31 +1438,40 @@
         <v>57</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="O1" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>38</v>
       </c>
@@ -1388,27 +1479,32 @@
       <c r="C2" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="9"/>
-      <c r="E2" s="8" t="s">
+      <c r="D2" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E2" s="9"/>
+      <c r="F2" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="8"/>
+      <c r="H2" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="8"/>
+      <c r="K2" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3"/>
+      <c r="M2" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="L2" s="3"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+    </row>
+    <row r="3" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>39</v>
       </c>
@@ -1416,27 +1512,32 @@
       <c r="C3" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8" t="s">
+      <c r="D3" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="8"/>
+      <c r="H3" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="I3" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="8"/>
+      <c r="K3" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3"/>
+      <c r="M3" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="L3" s="3"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+    </row>
+    <row r="4" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>42</v>
       </c>
@@ -1444,27 +1545,32 @@
       <c r="C4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="8" t="s">
+      <c r="D4" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="8"/>
+      <c r="H4" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="I4" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="8"/>
+      <c r="K4" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3"/>
+      <c r="M4" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="L4" s="3"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>43</v>
       </c>
@@ -1472,27 +1578,32 @@
       <c r="C5" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="8" t="s">
+      <c r="D5" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="8"/>
+      <c r="H5" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="8"/>
+      <c r="K5" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3" t="s">
+      <c r="L5" s="3"/>
+      <c r="M5" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="L5" s="3"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>45</v>
       </c>
@@ -1500,87 +1611,101 @@
       <c r="C6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>121</v>
       </c>
       <c r="J6" s="3"/>
       <c r="K6" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="L6" s="3"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="3"/>
+      <c r="F7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="3"/>
+      <c r="H7" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>122</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="L7" s="3"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="3"/>
+      <c r="H8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="I8" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
-    </row>
-    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+    </row>
+    <row r="9" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="3"/>
+      <c r="F9" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="F9" s="8"/>
       <c r="G9" s="8"/>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="8"/>
+      <c r="I9" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
+      <c r="J9" s="6"/>
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1593,32 +1718,33 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF4865F-6BB8-4976-9DE5-36DB3EE7176D}">
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
     <col min="2" max="2" width="31.7109375" customWidth="1"/>
     <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="24.140625" customWidth="1"/>
-    <col min="5" max="5" width="31" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" customWidth="1"/>
-    <col min="7" max="7" width="25.140625" customWidth="1"/>
-    <col min="8" max="8" width="30.28515625" customWidth="1"/>
-    <col min="9" max="9" width="21.7109375" customWidth="1"/>
-    <col min="10" max="10" width="37.7109375" customWidth="1"/>
-    <col min="11" max="11" width="27.140625" customWidth="1"/>
-    <col min="12" max="12" width="30.7109375" customWidth="1"/>
-    <col min="13" max="13" width="27.5703125" customWidth="1"/>
-    <col min="14" max="14" width="27.42578125" customWidth="1"/>
-    <col min="15" max="15" width="24.28515625" customWidth="1"/>
-    <col min="16" max="16" width="34.7109375" customWidth="1"/>
-    <col min="17" max="17" width="21.140625" customWidth="1"/>
-    <col min="18" max="18" width="33.140625" customWidth="1"/>
-    <col min="19" max="19" width="34.140625" customWidth="1"/>
-    <col min="20" max="20" width="32.28515625" customWidth="1"/>
+    <col min="4" max="5" width="24.140625" customWidth="1"/>
+    <col min="6" max="6" width="31" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" customWidth="1"/>
+    <col min="8" max="8" width="25.140625" customWidth="1"/>
+    <col min="9" max="10" width="30.28515625" customWidth="1"/>
+    <col min="11" max="11" width="21.7109375" customWidth="1"/>
+    <col min="12" max="12" width="37.7109375" customWidth="1"/>
+    <col min="13" max="13" width="27.140625" customWidth="1"/>
+    <col min="14" max="15" width="30.7109375" customWidth="1"/>
+    <col min="16" max="16" width="27.5703125" customWidth="1"/>
+    <col min="17" max="17" width="27.42578125" customWidth="1"/>
+    <col min="18" max="18" width="24.28515625" customWidth="1"/>
+    <col min="19" max="20" width="34.7109375" customWidth="1"/>
+    <col min="21" max="21" width="21.140625" customWidth="1"/>
+    <col min="22" max="22" width="33.140625" customWidth="1"/>
+    <col min="23" max="23" width="34.140625" customWidth="1"/>
+    <col min="24" max="24" width="32.28515625" customWidth="1"/>
+    <col min="25" max="25" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
@@ -1631,56 +1757,71 @@
       <c r="D1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="O1" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="T1" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="U1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="Y1" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>79</v>
       </c>
@@ -1693,50 +1834,55 @@
       <c r="D2" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="6"/>
+      <c r="F2" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="H2" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="J2" s="7"/>
+      <c r="K2" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8"/>
+      <c r="M2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="O2" s="8"/>
+      <c r="P2" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3" t="s">
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="S2" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="T2" s="3"/>
+      <c r="U2" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="R2" s="8"/>
-      <c r="S2" s="8" t="s">
+      <c r="V2" s="8"/>
+      <c r="W2" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="T2" s="8" t="s">
+      <c r="X2" s="8" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="Y2" s="3"/>
+    </row>
+    <row r="3" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>80</v>
       </c>
@@ -1749,50 +1895,55 @@
       <c r="D3" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="6"/>
+      <c r="F3" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>141</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>87</v>
       </c>
       <c r="J3" s="3"/>
       <c r="K3" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="O3" s="3"/>
+      <c r="P3" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8" t="s">
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="P3" s="8" t="s">
+      <c r="S3" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="T3" s="8"/>
+      <c r="U3" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3" t="s">
+      <c r="V3" s="3"/>
+      <c r="W3" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="X3" s="3" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="4" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+      <c r="Y3" s="3"/>
+    </row>
+    <row r="4" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>81</v>
       </c>
@@ -1805,109 +1956,119 @@
       <c r="D4" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="6"/>
+      <c r="F4" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>142</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>88</v>
       </c>
       <c r="J4" s="3"/>
       <c r="K4" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="L4" s="7" t="s">
+      <c r="N4" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="O4" s="7"/>
+      <c r="P4" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3" t="s">
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="P4" s="3" t="s">
+      <c r="S4" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="T4" s="3"/>
+      <c r="U4" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="R4" s="3"/>
-      <c r="S4" s="7" t="s">
+      <c r="V4" s="3"/>
+      <c r="W4" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="T4" s="7" t="s">
+      <c r="X4" s="7" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="5" spans="1:20" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y4" s="3"/>
+    </row>
+    <row r="5" spans="1:25" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
         <v>143</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>92</v>
       </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="N5" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="O5" s="7"/>
+      <c r="P5" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="N5" s="3"/>
-      <c r="O5" s="7" t="s">
+      <c r="Q5" s="3"/>
+      <c r="R5" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="S5" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="T5" s="7"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="3"/>
+      <c r="F6" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="I6" s="3"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
@@ -1919,8 +2080,14 @@
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
+      <c r="U6" s="3"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+      <c r="Y6" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1930,32 +2097,33 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73FA7BAE-C73F-432A-B85B-06103167559F}">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" customWidth="1"/>
     <col min="2" max="2" width="35.85546875" customWidth="1"/>
     <col min="3" max="3" width="34.28515625" customWidth="1"/>
-    <col min="4" max="4" width="37" customWidth="1"/>
-    <col min="5" max="5" width="30.5703125" customWidth="1"/>
-    <col min="6" max="6" width="31.140625" customWidth="1"/>
-    <col min="7" max="7" width="30.5703125" customWidth="1"/>
-    <col min="8" max="8" width="32.85546875" customWidth="1"/>
-    <col min="9" max="9" width="34.140625" customWidth="1"/>
-    <col min="10" max="10" width="31.140625" customWidth="1"/>
-    <col min="11" max="11" width="30.28515625" customWidth="1"/>
-    <col min="12" max="12" width="39.28515625" customWidth="1"/>
-    <col min="13" max="13" width="32.7109375" customWidth="1"/>
-    <col min="14" max="14" width="36.28515625" customWidth="1"/>
-    <col min="15" max="15" width="50.28515625" customWidth="1"/>
-    <col min="16" max="16" width="38.28515625" customWidth="1"/>
-    <col min="17" max="17" width="29.7109375" customWidth="1"/>
-    <col min="18" max="18" width="23.5703125" customWidth="1"/>
-    <col min="19" max="19" width="25.42578125" customWidth="1"/>
-    <col min="20" max="20" width="23" customWidth="1"/>
+    <col min="4" max="5" width="37" customWidth="1"/>
+    <col min="6" max="6" width="30.5703125" customWidth="1"/>
+    <col min="7" max="7" width="31.140625" customWidth="1"/>
+    <col min="8" max="8" width="30.5703125" customWidth="1"/>
+    <col min="9" max="10" width="32.85546875" customWidth="1"/>
+    <col min="11" max="11" width="34.140625" customWidth="1"/>
+    <col min="12" max="12" width="31.140625" customWidth="1"/>
+    <col min="13" max="13" width="30.28515625" customWidth="1"/>
+    <col min="14" max="15" width="39.28515625" customWidth="1"/>
+    <col min="16" max="16" width="32.7109375" customWidth="1"/>
+    <col min="17" max="17" width="36.28515625" customWidth="1"/>
+    <col min="18" max="18" width="50.28515625" customWidth="1"/>
+    <col min="19" max="20" width="38.28515625" customWidth="1"/>
+    <col min="21" max="21" width="29.7109375" customWidth="1"/>
+    <col min="22" max="22" width="23.5703125" customWidth="1"/>
+    <col min="23" max="23" width="25.42578125" customWidth="1"/>
+    <col min="24" max="24" width="23" customWidth="1"/>
+    <col min="25" max="25" width="21.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
@@ -1968,56 +2136,71 @@
       <c r="D1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="O1" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="T1" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="U1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="Y1" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>96</v>
       </c>
@@ -2028,48 +2211,53 @@
       <c r="D2" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6"/>
+      <c r="F2" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="7"/>
+      <c r="H2" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="7"/>
+      <c r="K2" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6" t="s">
+      <c r="L2" s="6"/>
+      <c r="M2" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="N2" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="O2" s="6"/>
+      <c r="P2" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7" t="s">
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="S2" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="T2" s="7"/>
+      <c r="U2" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6" t="s">
+      <c r="V2" s="6"/>
+      <c r="W2" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="T2" s="6" t="s">
+      <c r="X2" s="6" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+      <c r="Y2" s="7"/>
+    </row>
+    <row r="3" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>97</v>
       </c>
@@ -2080,94 +2268,105 @@
       <c r="D3" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6"/>
+      <c r="F3" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="7"/>
+      <c r="H3" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>157</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>102</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="N3" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="O3" s="7"/>
+      <c r="P3" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6" t="s">
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="S3" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="Q3" s="7" t="s">
+      <c r="T3" s="6"/>
+      <c r="U3" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="R3" s="7"/>
-      <c r="S3" s="7" t="s">
+      <c r="V3" s="7"/>
+      <c r="W3" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="T3" s="7" t="s">
+      <c r="X3" s="7" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="4" spans="1:20" ht="60" x14ac:dyDescent="0.25">
+      <c r="Y3" s="7"/>
+    </row>
+    <row r="4" spans="1:25" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="7"/>
+      <c r="F4" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="7"/>
+      <c r="H4" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>158</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>100</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="L4" s="7" t="s">
+      <c r="N4" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="O4" s="7"/>
+      <c r="P4" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7" t="s">
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="S4" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="Q4" s="7" t="s">
+      <c r="T4" s="7"/>
+      <c r="U4" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7" t="s">
+      <c r="V4" s="7"/>
+      <c r="W4" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="T4" s="7" t="s">
+      <c r="X4" s="7" t="s">
         <v>166</v>
       </c>
+      <c r="Y4" s="7"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
began on tech tree effect implementation
</commit_message>
<xml_diff>
--- a/Documentation/Tech tree.xlsx
+++ b/Documentation/Tech tree.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Documents\Final year uni\Comp-3000\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA5088E-B50C-48BC-9737-AA44FD676E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C623DA7-F623-45F9-9818-86C4764D71A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aspects of game" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="179">
   <si>
     <t>Core aspects</t>
   </si>
@@ -562,6 +562,9 @@
   </si>
   <si>
     <t>working on</t>
+  </si>
+  <si>
+    <t>Needs art</t>
   </si>
 </sst>
 </file>
@@ -1484,7 +1487,7 @@
         <v>173</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>44</v>
@@ -1499,7 +1502,7 @@
         <v>56</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>122</v>
@@ -1536,7 +1539,7 @@
         <v>58</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>123</v>
@@ -1573,7 +1576,7 @@
         <v>57</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>124</v>
@@ -1610,7 +1613,7 @@
         <v>63</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>117</v>
@@ -1733,8 +1736,8 @@
       <c r="I9" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="J9" s="5" t="s">
-        <v>177</v>
+      <c r="J9" s="7" t="s">
+        <v>178</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>

</xml_diff>

<commit_message>
adjust code to allow for easier modifing of values via tech tree
</commit_message>
<xml_diff>
--- a/Documentation/Tech tree.xlsx
+++ b/Documentation/Tech tree.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Documents\Final year uni\Comp-3000\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C623DA7-F623-45F9-9818-86C4764D71A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F338B99-4F4F-4672-9D69-249462866F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aspects of game" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="178">
   <si>
     <t>Core aspects</t>
   </si>
@@ -216,12 +216,6 @@
     <t>Ammo costs are decreased 10%</t>
   </si>
   <si>
-    <t>Scrap costs are decreased x3</t>
-  </si>
-  <si>
-    <t>Scrap costs are decreased 15%</t>
-  </si>
-  <si>
     <t>Pre-requisites</t>
   </si>
   <si>
@@ -565,6 +559,9 @@
   </si>
   <si>
     <t>Needs art</t>
+  </si>
+  <si>
+    <t>Needs rework</t>
   </si>
 </sst>
 </file>
@@ -1440,7 +1437,7 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>25</v>
@@ -1452,13 +1449,13 @@
         <v>32</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>35</v>
@@ -1467,15 +1464,15 @@
         <v>33</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B2" s="8">
         <v>50</v>
@@ -1484,16 +1481,16 @@
         <v>50</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>44</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H2" s="7" t="s">
         <v>50</v>
@@ -1502,10 +1499,10 @@
         <v>56</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
@@ -1523,14 +1520,14 @@
         <v>50</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="7" t="s">
         <v>45</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>50</v>
@@ -1539,14 +1536,14 @@
         <v>58</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -1560,14 +1557,14 @@
         <v>50</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="7" t="s">
         <v>46</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H4" s="7" t="s">
         <v>50</v>
@@ -1576,14 +1573,14 @@
         <v>57</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -1597,26 +1594,26 @@
         <v>40</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="F5" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>178</v>
+      <c r="F5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="2">
+        <v>200</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>177</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
@@ -1634,30 +1631,30 @@
         <v>40</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G6" s="2">
         <v>200</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>177</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -1669,26 +1666,26 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G7" s="2">
         <v>200</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>177</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1699,20 +1696,18 @@
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="2">
-        <v>200</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>177</v>
+      <c r="F8" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="H8" s="7"/>
+      <c r="I8" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>176</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
@@ -1726,19 +1721,11 @@
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="H9" s="7"/>
-      <c r="I9" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>178</v>
-      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
@@ -1791,13 +1778,13 @@
         <v>30</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>20</v>
@@ -1806,252 +1793,252 @@
         <v>35</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>21</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="O1" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>22</v>
       </c>
       <c r="Q1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="R1" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="T1" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>23</v>
       </c>
       <c r="V1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="X1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="W1" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="Y1" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>50</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>177</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L2" s="7"/>
       <c r="M2" s="7" t="s">
         <v>37</v>
       </c>
       <c r="N2" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="O2" s="7"/>
       <c r="P2" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="Q2" s="2"/>
       <c r="R2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="T2" s="2"/>
       <c r="U2" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="V2" s="7"/>
       <c r="W2" s="7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="X2" s="7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="Y2" s="2"/>
     </row>
     <row r="3" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>50</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>177</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
         <v>37</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="Q3" s="7"/>
       <c r="R3" s="7" t="s">
         <v>36</v>
       </c>
       <c r="S3" s="7" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="T3" s="7"/>
       <c r="U3" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="V3" s="2"/>
       <c r="W3" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="Y3" s="2"/>
     </row>
     <row r="4" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>50</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>177</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
         <v>37</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O4" s="6"/>
       <c r="P4" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q4" s="2"/>
       <c r="R4" s="2" t="s">
         <v>36</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="T4" s="2"/>
       <c r="U4" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="V4" s="2"/>
       <c r="W4" s="6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="X4" s="6" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="Y4" s="2"/>
     </row>
@@ -2062,40 +2049,40 @@
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="O5" s="6"/>
       <c r="P5" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="Q5" s="2"/>
       <c r="R5" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="T5" s="6"/>
       <c r="U5" s="2"/>
@@ -2111,19 +2098,19 @@
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -2186,13 +2173,13 @@
         <v>30</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>26</v>
@@ -2201,187 +2188,187 @@
         <v>35</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>27</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="O1" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>28</v>
       </c>
       <c r="Q1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="R1" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="T1" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>29</v>
       </c>
       <c r="V1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="X1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="W1" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="Y1" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>50</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G2" s="6">
         <v>200</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L2" s="5"/>
       <c r="M2" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="O2" s="5"/>
       <c r="P2" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="Q2" s="6"/>
       <c r="R2" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="T2" s="6"/>
       <c r="U2" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="Y2" s="6"/>
     </row>
     <row r="3" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>50</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>177</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G3" s="6">
         <v>200</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L3" s="6"/>
       <c r="M3" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="O3" s="6"/>
       <c r="P3" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="Q3" s="5"/>
       <c r="R3" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="T3" s="5"/>
       <c r="U3" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="V3" s="6"/>
       <c r="W3" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="X3" s="6" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="Y3" s="6"/>
     </row>
@@ -2392,51 +2379,51 @@
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G4" s="6">
         <v>200</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L4" s="6"/>
       <c r="M4" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="R4" s="6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="T4" s="6"/>
       <c r="U4" s="6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="V4" s="6"/>
       <c r="W4" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="X4" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="Y4" s="6"/>
     </row>

</xml_diff>

<commit_message>
did further work on implementing tech tree effects
</commit_message>
<xml_diff>
--- a/Documentation/Tech tree.xlsx
+++ b/Documentation/Tech tree.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Documents\Final year uni\Comp-3000\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F338B99-4F4F-4672-9D69-249462866F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1221EA3F-83B4-4330-8A2C-BB9D66B22261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="180">
   <si>
     <t>Core aspects</t>
   </si>
@@ -447,9 +447,6 @@
     <t>Rate of fire increase by 20%</t>
   </si>
   <si>
-    <t>Damage increase by 10%</t>
-  </si>
-  <si>
     <t>Movement speed increase by 5%</t>
   </si>
   <si>
@@ -562,6 +559,15 @@
   </si>
   <si>
     <t>Needs rework</t>
+  </si>
+  <si>
+    <t>Needs testing</t>
+  </si>
+  <si>
+    <t>Damage increase by 20%</t>
+  </si>
+  <si>
+    <t>needs testing</t>
   </si>
 </sst>
 </file>
@@ -1437,7 +1443,7 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>25</v>
@@ -1452,7 +1458,7 @@
         <v>125</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>114</v>
@@ -1467,12 +1473,12 @@
         <v>126</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B2" s="8">
         <v>50</v>
@@ -1481,16 +1487,16 @@
         <v>50</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>44</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H2" s="7" t="s">
         <v>50</v>
@@ -1499,7 +1505,7 @@
         <v>56</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>120</v>
@@ -1520,14 +1526,14 @@
         <v>50</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="7" t="s">
         <v>45</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>50</v>
@@ -1536,7 +1542,7 @@
         <v>58</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>121</v>
@@ -1557,14 +1563,14 @@
         <v>50</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="7" t="s">
         <v>46</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H4" s="7" t="s">
         <v>50</v>
@@ -1573,7 +1579,7 @@
         <v>57</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>122</v>
@@ -1594,7 +1600,7 @@
         <v>40</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
@@ -1610,7 +1616,7 @@
         <v>59</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>115</v>
@@ -1631,7 +1637,7 @@
         <v>40</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
@@ -1647,7 +1653,7 @@
         <v>60</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>116</v>
@@ -1678,7 +1684,7 @@
         <v>61</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>117</v>
@@ -1700,14 +1706,14 @@
         <v>54</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H8" s="7"/>
       <c r="I8" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
@@ -1784,7 +1790,7 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>20</v>
@@ -1799,7 +1805,7 @@
         <v>64</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>21</v>
@@ -1814,7 +1820,7 @@
         <v>67</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>22</v>
@@ -1829,7 +1835,7 @@
         <v>70</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>23</v>
@@ -1844,7 +1850,7 @@
         <v>73</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
@@ -1861,7 +1867,7 @@
         <v>132</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>77</v>
@@ -1876,7 +1882,7 @@
         <v>135</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K2" s="7" t="s">
         <v>81</v>
@@ -1886,7 +1892,7 @@
         <v>37</v>
       </c>
       <c r="N2" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O2" s="7"/>
       <c r="P2" s="2" t="s">
@@ -1897,7 +1903,7 @@
         <v>36</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="T2" s="2"/>
       <c r="U2" s="7" t="s">
@@ -1908,7 +1914,7 @@
         <v>105</v>
       </c>
       <c r="X2" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="Y2" s="2"/>
     </row>
@@ -1926,7 +1932,7 @@
         <v>133</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>78</v>
@@ -1941,7 +1947,7 @@
         <v>136</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>82</v>
@@ -1951,7 +1957,7 @@
         <v>37</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="7" t="s">
@@ -1962,7 +1968,7 @@
         <v>36</v>
       </c>
       <c r="S3" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="T3" s="7"/>
       <c r="U3" s="2" t="s">
@@ -1973,7 +1979,7 @@
         <v>105</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Y3" s="2"/>
     </row>
@@ -1991,7 +1997,7 @@
         <v>134</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>79</v>
@@ -2006,7 +2012,7 @@
         <v>137</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>83</v>
@@ -2016,7 +2022,7 @@
         <v>37</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O4" s="6"/>
       <c r="P4" s="2" t="s">
@@ -2027,7 +2033,7 @@
         <v>36</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="T4" s="2"/>
       <c r="U4" s="2" t="s">
@@ -2038,7 +2044,7 @@
         <v>106</v>
       </c>
       <c r="X4" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="Y4" s="2"/>
     </row>
@@ -2061,7 +2067,7 @@
         <v>138</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>87</v>
@@ -2071,7 +2077,7 @@
         <v>104</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O5" s="6"/>
       <c r="P5" s="2" t="s">
@@ -2082,7 +2088,7 @@
         <v>107</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="T5" s="6"/>
       <c r="U5" s="2"/>
@@ -2107,10 +2113,10 @@
         <v>103</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>139</v>
+        <v>178</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -2179,7 +2185,7 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>26</v>
@@ -2194,7 +2200,7 @@
         <v>64</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>27</v>
@@ -2209,7 +2215,7 @@
         <v>67</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>28</v>
@@ -2224,7 +2230,7 @@
         <v>70</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>29</v>
@@ -2239,7 +2245,7 @@
         <v>73</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
@@ -2247,16 +2253,16 @@
         <v>91</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>50</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>93</v>
@@ -2268,10 +2274,10 @@
         <v>103</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>96</v>
@@ -2281,7 +2287,7 @@
         <v>108</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="O2" s="5"/>
       <c r="P2" s="6" t="s">
@@ -2292,7 +2298,7 @@
         <v>110</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="T2" s="6"/>
       <c r="U2" s="5" t="s">
@@ -2303,7 +2309,7 @@
         <v>112</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="Y2" s="6"/>
     </row>
@@ -2312,7 +2318,7 @@
         <v>92</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>50</v>
@@ -2321,7 +2327,7 @@
         <v>133</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>94</v>
@@ -2333,10 +2339,10 @@
         <v>103</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K3" s="6" t="s">
         <v>97</v>
@@ -2346,7 +2352,7 @@
         <v>109</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="O3" s="6"/>
       <c r="P3" s="5" t="s">
@@ -2357,7 +2363,7 @@
         <v>110</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="T3" s="5"/>
       <c r="U3" s="6" t="s">
@@ -2368,7 +2374,7 @@
         <v>112</v>
       </c>
       <c r="X3" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Y3" s="6"/>
     </row>
@@ -2388,10 +2394,10 @@
         <v>103</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K4" s="6" t="s">
         <v>95</v>
@@ -2401,7 +2407,7 @@
         <v>108</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
@@ -2412,7 +2418,7 @@
         <v>111</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="T4" s="6"/>
       <c r="U4" s="6" t="s">
@@ -2423,7 +2429,7 @@
         <v>113</v>
       </c>
       <c r="X4" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Y4" s="6"/>
     </row>

</xml_diff>

<commit_message>
added icons to tech tree
</commit_message>
<xml_diff>
--- a/Documentation/Tech tree.xlsx
+++ b/Documentation/Tech tree.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Documents\Final year uni\Comp-3000\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1221EA3F-83B4-4330-8A2C-BB9D66B22261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E55B4D00-99BB-4CC1-B643-3E8F5D63455C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aspects of game" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="180">
   <si>
     <t>Core aspects</t>
   </si>
@@ -668,7 +668,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -691,6 +691,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2383,7 +2386,9 @@
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
+      <c r="E4" s="9" t="s">
+        <v>174</v>
+      </c>
       <c r="F4" s="6" t="s">
         <v>95</v>
       </c>

</xml_diff>

<commit_message>
fixed remaining techs that needs a rework
</commit_message>
<xml_diff>
--- a/Documentation/Tech tree.xlsx
+++ b/Documentation/Tech tree.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Documents\Final year uni\Comp-3000\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E55B4D00-99BB-4CC1-B643-3E8F5D63455C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A10DAC-14A3-4FBB-9E11-B75517A90D3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="4215" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aspects of game" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="180">
   <si>
     <t>Core aspects</t>
   </si>
@@ -865,73 +865,73 @@
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -947,37 +947,37 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7936B949-188E-4582-8616-623FBF3C46A1}" name="Table1" displayName="Table1" ref="A1:D6" totalsRowShown="0" headerRowDxfId="76" dataDxfId="75">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7936B949-188E-4582-8616-623FBF3C46A1}" name="Table1" displayName="Table1" ref="A1:D6" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
   <autoFilter ref="A1:D6" xr:uid="{7936B949-188E-4582-8616-623FBF3C46A1}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2EA6F07F-1C6E-40BA-AB5C-B295EB35CDCF}" name="Core aspects" dataDxfId="74"/>
-    <tableColumn id="2" xr3:uid="{194B2CAD-4A90-4E48-AEE8-DDC5F401A5C9}" name="Unit types" dataDxfId="73"/>
-    <tableColumn id="3" xr3:uid="{1448A4CC-616D-4E01-90A1-52101EAC6A7A}" name="Convoy types" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{B97AA103-9726-4AD2-A972-AE6976451B75}" name="Resources" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{2EA6F07F-1C6E-40BA-AB5C-B295EB35CDCF}" name="Core aspects" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{194B2CAD-4A90-4E48-AEE8-DDC5F401A5C9}" name="Unit types" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{1448A4CC-616D-4E01-90A1-52101EAC6A7A}" name="Convoy types" dataDxfId="55"/>
+    <tableColumn id="4" xr3:uid="{B97AA103-9726-4AD2-A972-AE6976451B75}" name="Resources" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}" name="Table4" displayName="Table4" ref="A1:O9" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}" name="Table4" displayName="Table4" ref="A1:O9" totalsRowShown="0" headerRowDxfId="76" dataDxfId="75">
   <autoFilter ref="A1:O9" xr:uid="{4B8BC961-7AD7-4C3B-AD78-4582E88561B3}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{273B543D-89B6-4955-A317-A6B9B4680CA3}" name="Defence upgrades" dataDxfId="68"/>
-    <tableColumn id="5" xr3:uid="{E2ECC974-9E12-4A07-BD63-BDCBEF1507C0}" name="Cost" dataDxfId="67"/>
-    <tableColumn id="6" xr3:uid="{2161316E-661A-4676-A677-BA66328341C0}" name="Pre-requsites" dataDxfId="66"/>
-    <tableColumn id="12" xr3:uid="{134C13E5-02FA-4F76-A06D-7102BADBA3D2}" name="Effect" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{08607D56-09F1-4FA2-99AF-93D77D869DF9}" name="Implemented" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{CF1CB81C-0620-4735-BF49-5EF70D5A95D0}" name="Resource upgrades" dataDxfId="63"/>
-    <tableColumn id="8" xr3:uid="{D99D59BE-3DBC-4DC5-AC81-B6150EC1D1F4}" name="Cost2" dataDxfId="62"/>
-    <tableColumn id="7" xr3:uid="{02031DC9-8EF0-41F2-9B6C-598F6108A5A8}" name="Pre-requsites2" dataDxfId="61"/>
-    <tableColumn id="11" xr3:uid="{1680DD95-5CE0-4B9B-8549-ACF0137CB507}" name="Effect2" dataDxfId="60"/>
-    <tableColumn id="14" xr3:uid="{6C98FEC6-2863-482A-A27B-066A0999E0FB}" name="Implemented2" dataDxfId="59"/>
-    <tableColumn id="3" xr3:uid="{7E8E2876-1732-4CE0-B4F5-8E46B994DD1E}" name="Unit/Convoy unlocks" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{F2927B2C-24A0-4651-8D25-5F857B914BCE}" name="Cost3" dataDxfId="57"/>
-    <tableColumn id="10" xr3:uid="{DA739A9E-7639-4351-9932-0344E3EFE921}" name="Pre-requsites3" dataDxfId="56"/>
-    <tableColumn id="15" xr3:uid="{1806C71A-ADC9-4BB5-A94B-CBDCF0FD8313}" name="Effect3" dataDxfId="55"/>
-    <tableColumn id="13" xr3:uid="{2CB92CE3-4985-4B3C-BB70-75B83BED998E}" name="Implemented3" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{273B543D-89B6-4955-A317-A6B9B4680CA3}" name="Defence upgrades" dataDxfId="74"/>
+    <tableColumn id="5" xr3:uid="{E2ECC974-9E12-4A07-BD63-BDCBEF1507C0}" name="Cost" dataDxfId="73"/>
+    <tableColumn id="6" xr3:uid="{2161316E-661A-4676-A677-BA66328341C0}" name="Pre-requsites" dataDxfId="72"/>
+    <tableColumn id="12" xr3:uid="{134C13E5-02FA-4F76-A06D-7102BADBA3D2}" name="Effect" dataDxfId="71"/>
+    <tableColumn id="4" xr3:uid="{08607D56-09F1-4FA2-99AF-93D77D869DF9}" name="Implemented" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{CF1CB81C-0620-4735-BF49-5EF70D5A95D0}" name="Resource upgrades" dataDxfId="69"/>
+    <tableColumn id="8" xr3:uid="{D99D59BE-3DBC-4DC5-AC81-B6150EC1D1F4}" name="Cost2" dataDxfId="68"/>
+    <tableColumn id="7" xr3:uid="{02031DC9-8EF0-41F2-9B6C-598F6108A5A8}" name="Pre-requsites2" dataDxfId="67"/>
+    <tableColumn id="11" xr3:uid="{1680DD95-5CE0-4B9B-8549-ACF0137CB507}" name="Effect2" dataDxfId="66"/>
+    <tableColumn id="14" xr3:uid="{6C98FEC6-2863-482A-A27B-066A0999E0FB}" name="Implemented2" dataDxfId="65"/>
+    <tableColumn id="3" xr3:uid="{7E8E2876-1732-4CE0-B4F5-8E46B994DD1E}" name="Unit/Convoy unlocks" dataDxfId="64"/>
+    <tableColumn id="9" xr3:uid="{F2927B2C-24A0-4651-8D25-5F857B914BCE}" name="Cost3" dataDxfId="63"/>
+    <tableColumn id="10" xr3:uid="{DA739A9E-7639-4351-9932-0344E3EFE921}" name="Pre-requsites3" dataDxfId="62"/>
+    <tableColumn id="15" xr3:uid="{1806C71A-ADC9-4BB5-A94B-CBDCF0FD8313}" name="Effect3" dataDxfId="61"/>
+    <tableColumn id="13" xr3:uid="{2CB92CE3-4985-4B3C-BB70-75B83BED998E}" name="Implemented3" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1619,7 +1619,7 @@
         <v>59</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>115</v>
@@ -1687,7 +1687,7 @@
         <v>61</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>117</v>
@@ -1935,7 +1935,7 @@
         <v>133</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>78</v>
@@ -2015,7 +2015,7 @@
         <v>137</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>83</v>
@@ -2330,7 +2330,7 @@
         <v>133</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>94</v>

</xml_diff>